<commit_message>
chore: fix tests + update excel highlights
</commit_message>
<xml_diff>
--- a/rules/CORE-000006/positive/01/data/unit-test-coreid-CG0131-positive.xlsx
+++ b/rules/CORE-000006/positive/01/data/unit-test-coreid-CG0131-positive.xlsx
@@ -614,7 +614,7 @@
           <t>DTHDTC</t>
         </is>
       </c>
-      <c r="L1" s="4" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>DTHFL</t>
         </is>
@@ -1090,7 +1090,7 @@
           <t>2021-02-18</t>
         </is>
       </c>
-      <c r="L5" s="9" t="inlineStr">
+      <c r="L5" s="7" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1214,7 +1214,7 @@
           <t>2021-11-25</t>
         </is>
       </c>
-      <c r="L6" s="9" t="inlineStr">
+      <c r="L6" s="7" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1338,7 +1338,7 @@
           <t>2018-09-04</t>
         </is>
       </c>
-      <c r="L7" s="9" t="inlineStr">
+      <c r="L7" s="7" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
@@ -1442,7 +1442,7 @@
         </is>
       </c>
       <c r="K8" s="8" t="n"/>
-      <c r="L8" s="9" t="n"/>
+      <c r="L8" s="7" t="n"/>
       <c r="M8" s="7" t="inlineStr">
         <is>
           <t>0360002</t>

</xml_diff>